<commit_message>
Claude OK 14/06/2026 03h00
</commit_message>
<xml_diff>
--- a/sites_20.xlsx
+++ b/sites_20.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zsavadogo\DevProject\Python\getBfSiteWebStatut\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B574735-5F9F-4261-BC19-0203D2420ABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A32384C-8251-40F7-B8F5-5EA0BF46FDED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{821148D1-6634-4CEC-A284-2D8B7EA34D13}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>▶ MINES / ÉNERGIE (16 domaines)</t>
   </si>
   <si>
-    <t>app.e-agrements.memc.gov.bf</t>
-  </si>
-  <si>
     <t>artisanminiersonasp.gov.bf</t>
   </si>
   <si>
@@ -126,6 +123,9 @@
   </si>
   <si>
     <t>Date de scan</t>
+  </si>
+  <si>
+    <t>eservices.cnss.bf</t>
   </si>
 </sst>
 </file>
@@ -661,28 +661,28 @@
   <sheetData>
     <row r="2" spans="1:12" s="10" customFormat="1" ht="46.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E2" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="G2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="I2" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="J2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="K2" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="L2" s="10" t="s">
         <v>28</v>
-      </c>
-      <c r="L2" s="10" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -696,7 +696,7 @@
         <v>720</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -704,7 +704,7 @@
         <v>721</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -712,7 +712,7 @@
         <v>722</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -720,7 +720,7 @@
         <v>723</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -728,7 +728,7 @@
         <v>724</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -736,7 +736,7 @@
         <v>725</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -744,7 +744,7 @@
         <v>726</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -752,7 +752,7 @@
         <v>727</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -760,7 +760,7 @@
         <v>728</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -768,7 +768,7 @@
         <v>729</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -776,7 +776,7 @@
         <v>730</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -784,7 +784,7 @@
         <v>731</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -792,7 +792,7 @@
         <v>732</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -800,7 +800,7 @@
         <v>733</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -808,7 +808,7 @@
         <v>734</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -816,13 +816,13 @@
         <v>735</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6"/>
       <c r="B20" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -830,7 +830,7 @@
         <v>736</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -838,7 +838,7 @@
         <v>737</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -846,7 +846,7 @@
         <v>738</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -854,7 +854,7 @@
         <v>739</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>